<commit_message>
update skill UI phải bám sát theo tài liệu
</commit_message>
<xml_diff>
--- a/log/作業ログ.xlsx
+++ b/log/作業ログ.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1779,6 +1779,92 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>L-027</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:30–16:45</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>BR_Com_004-WF-LAYOUT</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>User (chỉ thị), AI (thực hiện)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Workflow — đọc ảnh layout BD</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Hiệu chỉnh workflow</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh BD 会議室選択時 và ảnh màn hiện tại; skill 01-pg-guide, 02-pg, 03-reconcile; RUNBOOK; UI_RULES; template pg-guide</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện PG lệch BD (màu, icon, vị trí, độ dài ô) do skill không đọc ảnh レイアウト và tự suy đoán. Bổ sung bước trích và xem ảnh layout ở S1, triển khai và đối chiếu theo Layout spec ở S2/S3.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Copilot CLI, Claude Opus 5.5</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>python .agents/workflow/scripts/xlsx_media.py &lt;BD&gt; --out runs/BR_Com_004/inputs/layout (exit 0)</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Script mới xlsx_media.py (ảnh EMF→PNG + text shape); S1 bước 2a Layout spec bắt buộc, ảnh lỗi → hỏi user, PENDING; S2 bước 3a UI theo Layout spec + so ảnh; S3 kiểm UI; UI_RULES ưu tiên ảnh BD; template pg-guide 2a; RUNBOOK/README/WORKFLOW-START</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>User chốt: chỉ sửa component BR_Com_004, giữ theme/shell chung</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Script chạy thật trên BD004, trích đủ ảnh/shape</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Thành công</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Skill cũ cấm xin ảnh layout, chỉ ghi giới hạn</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R1"/>
   <dataValidations count="1">
@@ -1796,7 +1882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2951,6 +3037,92 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>L-028</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:35–16:50</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>BR_Com_004-S2-LAYOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>User (chỉ thị), AI (thực hiện)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>BR_Com_004 — S1 addendum + S2 UI</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Hiệu chỉnh thành phẩm</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>inputs/layout/image3.png, image9.png; br-com-004.component.{html,css}</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Restyle màn BR_Com_004 theo ảnh レイアウト của BD, chỉ trong component; bổ sung Layout spec vào pg-guide.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Copilot CLI, Claude Opus 5.5</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>prettier --check (pass); eslint (pass); tsc --noEmit (exit 0); ng build (pass); Edge headless chụp harness tĩnh</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>pg-guide 2a Layout spec; component CSS/HTML theo BD; pg-implementation P-21, D-10; source-manifest LAY01/LAY02</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>So ảnh chụp với image3 cả 2 state: khớp vị trí/màu/độ dài; shell giữ theme repo (D-10)</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Thành công</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Cần user review lại G0 (2a) và G1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R1"/>
   <dataValidations count="1">

</xml_diff>